<commit_message>
Ajouter fonctionalites/besoins au excel sprint 1
</commit_message>
<xml_diff>
--- a/Journal_de_sprint_equipe.xlsx
+++ b/Journal_de_sprint_equipe.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2249463\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{53AC90AF-038A-42CA-8C28-750CAAC43FCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4D6721DB-7B67-4A3A-97F7-474840700DBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="258" xr2:uid="{6BF6013A-4C68-4CEF-BF49-8F7071437FDB}"/>
   </bookViews>
@@ -887,9 +887,6 @@
     <t>Conception prototypes des 4 pages (Accueil, Inscription, Connexion, Abonnement) en html/css/js et Création compte qui s'insère dans la bdd</t>
   </si>
   <si>
-    <t>Pas de changement prévu</t>
-  </si>
-  <si>
     <t>Productivité, creativité, division des tâches, travail d'équipe</t>
   </si>
   <si>
@@ -900,6 +897,9 @@
   </si>
   <si>
     <t>N/A</t>
+  </si>
+  <si>
+    <t>Ajout de besoins et fonctionnalités : Utiliser un algorithme de machine learning pour faire les match des lieux des personnes, Ajouter un système de vérification de profil en utilisant une pièce d'identité</t>
   </si>
 </sst>
 </file>
@@ -1158,11 +1158,11 @@
     </xf>
   </cellXfs>
   <cellStyles count="5">
-    <cellStyle name="Calcul" xfId="4" builtinId="22"/>
-    <cellStyle name="Entrée" xfId="3" builtinId="20"/>
+    <cellStyle name="Calculation" xfId="4" builtinId="22"/>
+    <cellStyle name="Heading 2" xfId="1" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="2" builtinId="18"/>
+    <cellStyle name="Input" xfId="3" builtinId="20"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Titre 2" xfId="1" builtinId="17"/>
-    <cellStyle name="Titre 3" xfId="2" builtinId="18"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1499,7 +1499,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AE47C8C-BB64-4187-92AA-6B5ED698724D}">
   <dimension ref="A1:O39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="66.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
@@ -2053,16 +2053,16 @@
         <v>55</v>
       </c>
       <c r="L26" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="M26" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N26" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O26" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="27" spans="11:15" x14ac:dyDescent="0.25">
@@ -2070,16 +2070,16 @@
         <v>56</v>
       </c>
       <c r="L27" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="M27" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N27" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O27" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="30" spans="11:15" x14ac:dyDescent="0.25">
@@ -2103,7 +2103,7 @@
         <v>59</v>
       </c>
       <c r="L32" s="20" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="M32" s="20"/>
       <c r="N32" s="20"/>
@@ -2119,7 +2119,7 @@
         <v>61</v>
       </c>
       <c r="L35" s="20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="M35" s="20"/>
       <c r="N35" s="20"/>
@@ -2130,7 +2130,7 @@
         <v>62</v>
       </c>
       <c r="L36" s="20" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="M36" s="20"/>
       <c r="N36" s="20"/>
@@ -2141,7 +2141,7 @@
         <v>63</v>
       </c>
       <c r="L37" s="20" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="M37" s="20"/>
       <c r="N37" s="20"/>
@@ -2159,7 +2159,7 @@
         <v>64</v>
       </c>
       <c r="L39" s="20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="M39" s="20"/>
       <c r="N39" s="20"/>

</xml_diff>